<commit_message>
updating for test 25-02-26
</commit_message>
<xml_diff>
--- a/client posts status.xlsx
+++ b/client posts status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\client posting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F50CBC-A35D-42A0-98E2-D15609E0F9A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F429BB76-A34F-4E40-AB1E-06324B56E120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FF3F5B0C-C890-4C84-898F-5F723B2BFDE4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="24">
   <si>
     <t xml:space="preserve">content title </t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>test 2</t>
   </si>
 </sst>
 </file>
@@ -742,7 +745,9 @@
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
+      <c r="A11" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>

</xml_diff>

<commit_message>
updated on 25-02-2026 time:4:27pm
</commit_message>
<xml_diff>
--- a/client posts status.xlsx
+++ b/client posts status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\client posting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DCA573-2AC3-49A0-B15B-52FE3737638C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5184C3C-8C84-4CDF-8170-F71075100E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FF3F5B0C-C890-4C84-898F-5F723B2BFDE4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="29">
   <si>
     <t xml:space="preserve">content title </t>
   </si>
@@ -122,7 +122,7 @@
     <t>not received the poster</t>
   </si>
   <si>
-    <t>pending - received content today</t>
+    <t>reel received 25-02-2026</t>
   </si>
 </sst>
 </file>
@@ -729,9 +729,11 @@
       <c r="D8" s="2">
         <v>46076</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2">
+        <v>46078</v>
+      </c>
       <c r="F8" s="9" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="G8" s="1"/>
     </row>
@@ -792,7 +794,9 @@
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
+      <c r="G11" s="9" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="12" spans="1:14" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">

</xml_diff>

<commit_message>
updated on 25-02-2026 time:08:47pm
</commit_message>
<xml_diff>
--- a/client posts status.xlsx
+++ b/client posts status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\client posting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5184C3C-8C84-4CDF-8170-F71075100E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC683A9D-73E5-4EDE-BFEF-013800EB429C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FF3F5B0C-C890-4C84-898F-5F723B2BFDE4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="28">
   <si>
     <t xml:space="preserve">content title </t>
   </si>
@@ -117,9 +117,6 @@
   </si>
   <si>
     <t>reel and poster</t>
-  </si>
-  <si>
-    <t>not received the poster</t>
   </si>
   <si>
     <t>reel received 25-02-2026</t>
@@ -771,13 +768,13 @@
       <c r="D10" s="2">
         <v>46105</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="2">
+        <v>46078</v>
+      </c>
       <c r="F10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -795,7 +792,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated on 26th feb 2026
</commit_message>
<xml_diff>
--- a/client posts status.xlsx
+++ b/client posts status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\client posting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC683A9D-73E5-4EDE-BFEF-013800EB429C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139D3AC2-5C5F-47F5-AA26-B6C469132E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FF3F5B0C-C890-4C84-898F-5F723B2BFDE4}"/>
   </bookViews>
@@ -113,13 +113,13 @@
     <t>portico</t>
   </si>
   <si>
-    <t>yet to post - need to change the password of social media</t>
-  </si>
-  <si>
     <t>reel and poster</t>
   </si>
   <si>
-    <t>reel received 25-02-2026</t>
+    <t xml:space="preserve">reel received (chest pain) </t>
+  </si>
+  <si>
+    <t>reel received - yet to post - need to change the password of social media</t>
   </si>
 </sst>
 </file>
@@ -556,7 +556,7 @@
     <col min="4" max="4" width="26.33203125" customWidth="1"/>
     <col min="5" max="5" width="21.5546875" customWidth="1"/>
     <col min="6" max="6" width="19.33203125" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="4" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.3">
@@ -608,7 +608,6 @@
       <c r="F2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -629,7 +628,6 @@
       <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:14" s="7" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -671,7 +669,6 @@
       <c r="F5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -690,7 +687,6 @@
       <c r="F6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -711,7 +707,6 @@
       <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -732,7 +727,6 @@
       <c r="F8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:14" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -752,7 +746,7 @@
         <v>18</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -774,7 +768,6 @@
       <c r="F10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -791,9 +784,7 @@
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="9" t="s">
-        <v>27</v>
-      </c>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:14" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
@@ -810,13 +801,16 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
+      <c r="G12" s="9" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="13" spans="1:14" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>17</v>

</xml_diff>